<commit_message>
Corrige cantidades con datos reales del plano: excavacion desplante 1.5m, subbase 0.30m, columnetas c/1.5m (total $218.3M)
</commit_message>
<xml_diff>
--- a/Proyectos/Fundamentos-de-Construccion/Solucion/CARTILLA DE HIERROS - despiece CDI TESALIA.xlsx
+++ b/Proyectos/Fundamentos-de-Construccion/Solucion/CARTILLA DE HIERROS - despiece CDI TESALIA.xlsx
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>168.2</v>
+        <v>336.4</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>4</v>
@@ -1084,7 +1084,7 @@
         <v>0.5</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>841</v>
+        <v>1682</v>
       </c>
       <c r="G17" s="5" t="n">
         <v>1</v>
@@ -1205,7 +1205,7 @@
       <c r="H24" s="14" t="n"/>
       <c r="I24" s="14" t="n"/>
       <c r="J24" s="7" t="n">
-        <v>530.1</v>
+        <v>1031.7</v>
       </c>
     </row>
     <row r="25">
@@ -1259,7 +1259,7 @@
       <c r="H27" s="16" t="n"/>
       <c r="I27" s="16" t="n"/>
       <c r="J27" s="17" t="n">
-        <v>6418</v>
+        <v>6919.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrige columnas (8 und, 2 secciones 0.50 y 0.40), zapatas reales Z-1/Z-2, altura muro 3.0m y excavacion por pozos+zanjas (total $215.9M)
</commit_message>
<xml_diff>
--- a/Proyectos/Fundamentos-de-Construccion/Solucion/CARTILLA DE HIERROS - despiece CDI TESALIA.xlsx
+++ b/Proyectos/Fundamentos-de-Construccion/Solucion/CARTILLA DE HIERROS - despiece CDI TESALIA.xlsx
@@ -755,7 +755,7 @@
         <v>2</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H8" s="7">
         <f>E8*F8*G8</f>
@@ -797,7 +797,7 @@
         <v>2</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H9" s="7">
         <f>E9*F9*G9</f>
@@ -839,7 +839,7 @@
         <v>24</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H10" s="7">
         <f>E10*F10*G10</f>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>336.4</v>
+        <v>348</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>4</v>
@@ -1084,7 +1084,7 @@
         <v>0.5</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>1682</v>
+        <v>1740</v>
       </c>
       <c r="G17" s="5" t="n">
         <v>1</v>
@@ -1169,7 +1169,7 @@
       <c r="H22" s="14" t="n"/>
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="7" t="n">
-        <v>791.8</v>
+        <v>644.2</v>
       </c>
     </row>
     <row r="23">
@@ -1205,7 +1205,7 @@
       <c r="H24" s="14" t="n"/>
       <c r="I24" s="14" t="n"/>
       <c r="J24" s="7" t="n">
-        <v>1031.7</v>
+        <v>1067.2</v>
       </c>
     </row>
     <row r="25">
@@ -1259,7 +1259,7 @@
       <c r="H27" s="16" t="n"/>
       <c r="I27" s="16" t="n"/>
       <c r="J27" s="17" t="n">
-        <v>6919.6</v>
+        <v>6807.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>